<commit_message>
Added landfill process to ODYM config file
</commit_message>
<xml_diff>
--- a/docs/Files/ODYM_Config_Tutorial6LL.xlsx
+++ b/docs/Files/ODYM_Config_Tutorial6LL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elanphear\Code\ODYM\docs\Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B53EB33-D91F-44BE-805F-239DD5336436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E86946D-76A8-43BC-9B32-374ED5D5DC8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="132">
   <si>
     <t>Description</t>
   </si>
@@ -427,6 +427,9 @@
   </si>
   <si>
     <t>[1,3,6,8,9,13,15,25,26,27,28,29]</t>
+  </si>
+  <si>
+    <t>Landfill</t>
   </si>
 </sst>
 </file>
@@ -996,14 +999,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.54296875" customWidth="1"/>
+    <col min="4" max="4" width="26.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B1" s="29" t="s">
         <v>38</v>
       </c>
@@ -1011,7 +1014,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="6"/>
       <c r="B2" s="8" t="s">
         <v>40</v>
@@ -1021,12 +1024,12 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6"/>
       <c r="B3" s="8"/>
       <c r="C3" s="3"/>
     </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6"/>
       <c r="B4" s="9" t="s">
         <v>2</v>
@@ -1037,7 +1040,7 @@
       </c>
       <c r="G4" s="35"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="B5" s="9" t="s">
         <v>55</v>
@@ -1051,122 +1054,122 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>
       <c r="B6" s="9"/>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="9"/>
       <c r="C7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="9"/>
       <c r="C8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="11"/>
       <c r="C9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="10"/>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
       <c r="B11" s="12"/>
       <c r="C11" s="14"/>
       <c r="D11" s="12"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="10"/>
       <c r="B12" s="12"/>
       <c r="C12" s="15"/>
       <c r="D12" s="12"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="10"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="10"/>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="10"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="10"/>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="10"/>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="10"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="10"/>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="10"/>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="10"/>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="10"/>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="6"/>
       <c r="B25" s="1"/>
       <c r="C25" s="2"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="6"/>
       <c r="B26" s="1"/>
       <c r="C26" s="2"/>
@@ -1179,20 +1182,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:J59"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B2:J60"/>
+  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="4.81640625" customWidth="1"/>
+    <col min="2" max="2" width="4.77734375" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="44.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.6328125" customWidth="1"/>
-    <col min="6" max="6" width="24.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.6328125" customWidth="1"/>
-    <col min="8" max="8" width="20.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" customWidth="1"/>
+    <col min="6" max="6" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.6640625" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" s="18" t="s">
         <v>3</v>
       </c>
@@ -1203,7 +1206,7 @@
       <c r="G2" s="19"/>
       <c r="H2" s="20"/>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C3" s="23" t="s">
         <v>27</v>
       </c>
@@ -1215,7 +1218,7 @@
       <c r="G3" s="30"/>
       <c r="H3" s="30"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>4</v>
       </c>
@@ -1223,7 +1226,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>0</v>
       </c>
@@ -1231,7 +1234,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>5</v>
       </c>
@@ -1239,11 +1242,11 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="D7" s="7"/>
       <c r="J7" s="13"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B8" s="18" t="s">
         <v>41</v>
       </c>
@@ -1255,7 +1258,7 @@
       <c r="H8" s="20"/>
       <c r="J8" s="13"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C9" s="23" t="s">
         <v>27</v>
       </c>
@@ -1270,7 +1273,7 @@
       <c r="H9" s="30"/>
       <c r="J9" s="13"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
         <v>6</v>
       </c>
@@ -1279,7 +1282,7 @@
       </c>
       <c r="J10" s="13"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
         <v>60</v>
       </c>
@@ -1288,7 +1291,7 @@
       </c>
       <c r="J11" s="13"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C12" t="s">
         <v>61</v>
       </c>
@@ -1297,10 +1300,10 @@
       </c>
       <c r="J12" s="13"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
       <c r="J13" s="17"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B14" s="18" t="s">
         <v>53</v>
       </c>
@@ -1313,7 +1316,7 @@
       <c r="G14" s="19"/>
       <c r="H14" s="20"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C15" s="24" t="s">
         <v>7</v>
       </c>
@@ -1339,7 +1342,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C16" s="25" t="s">
         <v>11</v>
       </c>
@@ -1362,7 +1365,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C17" s="25" t="s">
         <v>76</v>
       </c>
@@ -1385,7 +1388,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C18" s="25" t="s">
         <v>15</v>
       </c>
@@ -1408,7 +1411,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C19" s="25" t="s">
         <v>16</v>
       </c>
@@ -1431,7 +1434,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C20" s="25" t="s">
         <v>82</v>
       </c>
@@ -1454,7 +1457,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C21" s="25" t="s">
         <v>63</v>
       </c>
@@ -1477,7 +1480,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C22" s="25" t="s">
         <v>12</v>
       </c>
@@ -1500,7 +1503,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C23" s="25" t="s">
         <v>14</v>
       </c>
@@ -1523,7 +1526,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C24" s="21" t="s">
         <v>92</v>
       </c>
@@ -1546,7 +1549,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B26" s="18" t="s">
         <v>49</v>
       </c>
@@ -1557,7 +1560,7 @@
       <c r="G26" s="19"/>
       <c r="H26" s="20"/>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C27" s="26" t="s">
         <v>50</v>
       </c>
@@ -1573,7 +1576,7 @@
       <c r="G27" s="30"/>
       <c r="H27" s="30"/>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C28" s="31">
         <v>0</v>
       </c>
@@ -1584,7 +1587,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C29" s="31">
         <v>1</v>
       </c>
@@ -1595,7 +1598,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C30" s="27">
         <v>2</v>
       </c>
@@ -1606,7 +1609,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C31" s="27">
         <v>3</v>
       </c>
@@ -1617,7 +1620,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C32" s="31">
         <v>4</v>
       </c>
@@ -1628,7 +1631,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C33" s="27">
         <v>5</v>
       </c>
@@ -1639,7 +1642,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C34" s="31">
         <v>6</v>
       </c>
@@ -1650,7 +1653,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C35" s="27">
         <v>7</v>
       </c>
@@ -1661,7 +1664,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C36" s="31">
         <v>8</v>
       </c>
@@ -1672,98 +1675,86 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B38" s="18" t="s">
+    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C37" s="31">
+        <v>9</v>
+      </c>
+      <c r="D37" t="s">
+        <v>131</v>
+      </c>
+      <c r="E37" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B39" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="20"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="C39" s="26" t="s">
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="19"/>
+      <c r="H39" s="20"/>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C40" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="D39" s="23" t="s">
+      <c r="D40" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="E39" s="23" t="s">
+      <c r="E40" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="F39" s="23" t="s">
+      <c r="F40" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="G39" s="39" t="s">
+      <c r="G40" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="H39" s="23" t="s">
+      <c r="H40" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="I39" s="36" t="s">
+      <c r="I40" s="36" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="C40" t="s">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C41" t="s">
         <v>117</v>
       </c>
-      <c r="D40" s="38" t="s">
+      <c r="D41" s="38" t="s">
         <v>124</v>
-      </c>
-      <c r="E40" t="s">
-        <v>97</v>
-      </c>
-      <c r="F40" t="s">
-        <v>64</v>
-      </c>
-      <c r="G40" t="s">
-        <v>31</v>
-      </c>
-      <c r="H40" t="s">
-        <v>31</v>
-      </c>
-      <c r="I40" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="C41" s="27" t="s">
-        <v>126</v>
-      </c>
-      <c r="D41" t="s">
-        <v>128</v>
       </c>
       <c r="E41" t="s">
         <v>97</v>
       </c>
       <c r="F41" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
       <c r="G41" t="s">
-        <v>81</v>
+        <v>31</v>
       </c>
       <c r="H41" t="s">
         <v>31</v>
       </c>
       <c r="I41" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.35">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C42" s="27" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="D42" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E42" t="s">
         <v>97</v>
       </c>
       <c r="F42" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G42" t="s">
         <v>81</v>
@@ -1771,16 +1762,16 @@
       <c r="H42" t="s">
         <v>31</v>
       </c>
-      <c r="I42" s="37" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="I42" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C43" s="27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D43" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="E43" t="s">
         <v>97</v>
@@ -1795,41 +1786,44 @@
         <v>31</v>
       </c>
       <c r="I43" s="37" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.35">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C44" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D44" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E44" t="s">
         <v>97</v>
       </c>
       <c r="F44" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G44" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="H44" t="s">
         <v>31</v>
       </c>
       <c r="I44" s="37" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C45" s="27" t="s">
-        <v>121</v>
+        <v>120</v>
+      </c>
+      <c r="D45" t="s">
+        <v>108</v>
       </c>
       <c r="E45" t="s">
         <v>97</v>
       </c>
       <c r="F45" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="G45" t="s">
         <v>86</v>
@@ -1838,80 +1832,100 @@
         <v>31</v>
       </c>
       <c r="I45" s="37" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C46" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="E46" t="s">
+        <v>97</v>
+      </c>
+      <c r="F46" t="s">
+        <v>110</v>
+      </c>
+      <c r="G46" t="s">
+        <v>86</v>
+      </c>
+      <c r="H46" t="s">
+        <v>31</v>
+      </c>
+      <c r="I46" s="37" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="C46" s="27"/>
-    </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B47" s="18" t="s">
+    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C47" s="27"/>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B48" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="19"/>
-      <c r="F47" s="19"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="20"/>
-    </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="C48" t="s">
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="19"/>
+      <c r="G48" s="19"/>
+      <c r="H48" s="20"/>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C49" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="C49" s="27" t="s">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C50" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="D49" s="33" t="s">
+      <c r="D50" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E50" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="D50" s="33"/>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
       <c r="D51" s="33"/>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
       <c r="D52" s="33"/>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
       <c r="D53" s="33"/>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
       <c r="D54" s="33"/>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B56" s="18" t="s">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="D55" s="33"/>
+    </row>
+    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B57" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C56" s="19"/>
-      <c r="D56" s="19"/>
-      <c r="E56" s="19"/>
-      <c r="F56" s="19"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="20"/>
-    </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="C57" t="s">
+      <c r="C57" s="19"/>
+      <c r="D57" s="19"/>
+      <c r="E57" s="19"/>
+      <c r="F57" s="19"/>
+      <c r="G57" s="19"/>
+      <c r="H57" s="20"/>
+    </row>
+    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C58" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B59" s="18" t="s">
+    <row r="60" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B60" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="C59" s="19"/>
-      <c r="D59" s="19"/>
-      <c r="E59" s="19"/>
-      <c r="F59" s="19"/>
-      <c r="G59" s="19"/>
-      <c r="H59" s="20"/>
+      <c r="C60" s="19"/>
+      <c r="D60" s="19"/>
+      <c r="E60" s="19"/>
+      <c r="F60" s="19"/>
+      <c r="G60" s="19"/>
+      <c r="H60" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>